<commit_message>
Update agriculture Excel files from version 21 to 58 with various changes
</commit_message>
<xml_diff>
--- a/agriculture 21.xlsx
+++ b/agriculture 21.xlsx
@@ -133,7 +133,7 @@
     <t xml:space="preserve"> 2019-20</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit:- Percentage(%)</t>
+    <t xml:space="preserve">Unit:- Percentage (%)</t>
   </si>
   <si>
     <t xml:space="preserve">Source: Directorate of Economics and Statistics (1998-2020)</t>
@@ -315,7 +315,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB25"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="46.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">

</xml_diff>